<commit_message>
Use Copilot direct edits across Labs 2-6
</commit_message>
<xml_diff>
--- a/labs/lab-2/downloads/Project_Atlas_Field_Level_Action_Register.xlsx
+++ b/labs/lab-2/downloads/Project_Atlas_Field_Level_Action_Register.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="Rdda162ed2eea46ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Action Register" sheetId="2" r:id="Rad7ac78e24574d38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Change Queue" sheetId="3" r:id="Ra054ff9a02444cd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="New Action Queue" sheetId="4" r:id="R24c2c745d8e24ba9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Before Snapshot" sheetId="5" r:id="R41b12f1fce544790"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Before-After Audit" sheetId="6" r:id="R17e0b737627f4dda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation" sheetId="7" r:id="R9b3c0ad751594058"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R4426b8b11cc44ab6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Action Register" sheetId="2" r:id="R35199a5e5c4d4b5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Change Queue" sheetId="3" r:id="R6fea608c454444cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="New Action Queue" sheetId="4" r:id="R909b59ba3110424e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Before Snapshot" sheetId="5" r:id="R35bc8925a34240cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Before-After Audit" sheetId="6" r:id="R0068436ecd8844ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation" sheetId="7" r:id="R4226fed07a654c35"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -910,7 +910,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B10" s="35" t="str">
-        <x:v>Extract candidate changes in Copilot Chat</x:v>
+        <x:v>Use Copilot in Excel Edit mode</x:v>
       </x:c>
       <x:c r="C10" s="35" t="str">
         <x:v>Field-level proposed delta</x:v>
@@ -922,13 +922,13 @@
         <x:v>7 min</x:v>
       </x:c>
       <x:c r="F10" s="35" t="str">
-        <x:v>Meeting Notes</x:v>
+        <x:v>Meeting Notes + Action Register</x:v>
       </x:c>
       <x:c r="G10" s="35" t="str">
-        <x:v>Field Change Queue</x:v>
+        <x:v>Copilot writes to Field Change Queue</x:v>
       </x:c>
       <x:c r="H10" s="35" t="str">
-        <x:v>No full-row update is proposed</x:v>
+        <x:v>Target range reviewed before Apply</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -936,7 +936,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B11" s="35" t="str">
-        <x:v>Compare every proposal with Excel</x:v>
+        <x:v>Ask Copilot to populate both queues</x:v>
       </x:c>
       <x:c r="C11" s="35" t="str">
         <x:v>Current and proposed values</x:v>
@@ -948,13 +948,13 @@
         <x:v>8 min</x:v>
       </x:c>
       <x:c r="F11" s="35" t="str">
-        <x:v>Action Register</x:v>
+        <x:v>Both sources</x:v>
       </x:c>
       <x:c r="G11" s="35" t="str">
-        <x:v>Field Change Queue</x:v>
+        <x:v>Field Change Queue + New Action Queue</x:v>
       </x:c>
       <x:c r="H11" s="35" t="str">
-        <x:v>Matches use Action IDs</x:v>
+        <x:v>No manual transfer; matches use Action IDs</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -2059,7 +2059,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39e0d77db49249a6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf354d0b6c3544f73"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2394,7 +2394,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra883a3486d6544c9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae1867ca4090444f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2669,7 +2669,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c26d59f610d4a92"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf778f9f246543cd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3029,7 +3029,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31661aa9655c4d86"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06ece880357f4ced"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3369,7 +3369,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9436f627b9aa4c30"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R740103dfd5e64df8"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>